<commit_message>
regenerate file using the updated code
</commit_message>
<xml_diff>
--- a/data/raw/RPi_4_BoM_Official.xlsx
+++ b/data/raw/RPi_4_BoM_Official.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\szb75\Documents\Other_Proj\ArchitecturalCarbonModelingTool\ACT\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{977AC32B-A777-45A3-8AF5-FA423C08DDA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25EB5893-37B5-4DC2-A1EF-97ECFF38796D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{5023E1F4-0389-4A9C-A1C1-8A547001B1C6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5023E1F4-0389-4A9C-A1C1-8A547001B1C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -104,7 +104,9 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    ?</t>
+    ?
+Reply:
+    General passive</t>
       </text>
     </comment>
     <comment ref="C73" authorId="1" shapeId="0" xr:uid="{73A60986-AA6F-482B-84A1-F6B4563EBC6C}">
@@ -127,7 +129,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="253">
   <si>
     <t>Quantity</t>
   </si>
@@ -1626,6 +1628,9 @@
   <threadedComment ref="D50" dT="2026-03-05T03:58:49.09" personId="{0F8F5534-B3F4-405E-985E-75D8CCDF5EA7}" id="{8098779F-A106-4649-BC46-225A24C398C3}">
     <text>?</text>
   </threadedComment>
+  <threadedComment ref="D50" dT="2026-03-05T20:46:41.03" personId="{0F8F5534-B3F4-405E-985E-75D8CCDF5EA7}" id="{B904FBBF-1A9D-4096-BA53-23C691BF42B7}" parentId="{8098779F-A106-4649-BC46-225A24C398C3}">
+    <text>General passive</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -3136,9 +3141,7 @@
       <c r="B45" s="23">
         <v>6</v>
       </c>
-      <c r="C45" s="24" t="s">
-        <v>65</v>
-      </c>
+      <c r="C45" s="24"/>
       <c r="D45" s="25" t="s">
         <v>24</v>
       </c>
@@ -3296,7 +3299,9 @@
       <c r="D50" s="55" t="s">
         <v>132</v>
       </c>
-      <c r="E50" s="25"/>
+      <c r="E50" s="25" t="s">
+        <v>247</v>
+      </c>
       <c r="F50" s="26" t="s">
         <v>133</v>
       </c>
@@ -3314,7 +3319,9 @@
       <c r="L50" s="19"/>
       <c r="M50" s="19"/>
       <c r="N50" s="19"/>
-      <c r="O50" s="19"/>
+      <c r="O50" s="19" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="51" spans="2:15" ht="38.5" x14ac:dyDescent="0.35">
       <c r="B51" s="23">

</xml_diff>